<commit_message>
Add lead results 2026-10-02
</commit_message>
<xml_diff>
--- a/results/AceAds-DM-outreach-Wedding-Photo-Video-QLD.xlsx
+++ b/results/AceAds-DM-outreach-Wedding-Photo-Video-QLD.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to work this list" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$S$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$S$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,17 +49,12 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -84,9 +79,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -98,10 +93,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -501,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -628,22 +620,22 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>VERIFY FIRST</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>No website found</t>
+          <t>Weak website</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Sonja Griffioen - Newborn Photography</t>
+          <t>The Light Photo and Film</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>photographer</t>
+          <t>wedding photo or video</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -653,29 +645,29 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/sonjagriffioen.newborns/</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>+61 426 987 722</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr"/>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/thelight.photoandfilm</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>https://thelightphotoandfilm.com.au/</t>
+        </is>
+      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>no website listed, only social media (verify on Google Maps)</t>
+          <t>slow to load (3.7s)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Hi Sonja Griffioen - Newborn Photography team! [one real detail from their page]. We're AceAds, a web design studio. We couldn't find a website for Sonja Griffioen - Newborn Photography, only your Facebook. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+          <t>Hi The Light Photo and Film team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
@@ -697,7 +689,7 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -709,12 +701,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Wingman Media</t>
+          <t>Verona Media</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>photographer</t>
+          <t>wedding photo or video</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -724,23 +716,23 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/verona_media</t>
+        </is>
+      </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/WingmanMediaAustralia</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>+61 424 075 002</t>
-        </is>
-      </c>
+          <t>https://www.facebook.com/veronamedia</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>https://wingmanmedia.com.au/</t>
+          <t>https://www.veronamedia.com.au/</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -750,7 +742,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Hi Wingman Media team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+          <t>Hi Verona Media team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
@@ -772,7 +764,7 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -784,12 +776,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Zoo Studio</t>
+          <t>A Thousand Miles Photography</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>photographer</t>
+          <t>wedding photographer</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -799,37 +791,29 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/zoostudiophotos</t>
-        </is>
-      </c>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>http://www.facebook.com/ZooStudioPhotography</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>+61 7 3870 0903</t>
-        </is>
-      </c>
+          <t>https://www.facebook.com/athousandmilesphotography</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>https://www.zoostudio.com.au/</t>
+          <t>https://www.athousandmilesphotography.com.au/</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>slow to load (6.9s)</t>
+          <t>looks outdated (copyright 2022); slow to load (3.1s)</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Hi Zoo Studio team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+          <t>Hi A Thousand Miles Photography team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
@@ -851,7 +835,7 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -863,17 +847,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Heritage City Photos</t>
+          <t>Alison Cooke Photography</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>photographer</t>
+          <t>wedding photographer</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Brisbane</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -883,32 +867,28 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/heritagecityphotos2</t>
+          <t>https://www.instagram.com/alisoncookephotography</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/heritagecityphotos</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>+61 7 3202 3097</t>
-        </is>
-      </c>
+          <t>https://www.facebook.com/alisoncookephotographybrisbane</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>https://heritagecityphotos.com.au/</t>
+          <t>https://alisoncookephotography.com/</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>slow to load (6.1s)</t>
+          <t>looks outdated (copyright 2020)</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Hi Heritage City Photos team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+          <t>Hi Alison Cooke Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -930,7 +910,7 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -942,17 +922,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Korsos Photography</t>
+          <t>Willidea Studio</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>photographer</t>
+          <t>wedding photographer</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sunshine Coast</t>
+          <t>Brisbane</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -962,32 +942,28 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/korsosphotography</t>
+          <t>https://www.instagram.com/willideastudio</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/korsosphotography</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>+61 7 5373 7619</t>
-        </is>
-      </c>
+          <t>https://www.facebook.com/willideastudio</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>https://www.korsos.com.au</t>
+          <t>https://willidea.net/</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>looks outdated (copyright 2020); slow to load (4.3s)</t>
+          <t>slow to load (4.5s)</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Hi Korsos Photography team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+          <t>Hi Willidea Studio team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -1005,9 +981,1651 @@
       <c r="R6" s="2" t="inlineStr"/>
       <c r="S6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Nikki Blades Photography</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Bundaberg</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nikki_blades_photos</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/NikkiBladesPhotos</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nikkibladesphotography.com.au/</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2017); missing meta description; slow to load (4.1s)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Hi Nikki Blades Photography team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Sharon Dawn Photography</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Bundaberg</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>https://instagram.com/sharondawnphotography</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/sharondawnphotography</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>https://sharondawnphotography.queensberryworkspace.com/</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2021)</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Hi Sharon Dawn Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Lifetime in a Day Films</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>wedding videographer</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Bundaberg</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lifetime_in_a_day_films</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/lifetimeinaday</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>https://lifetimeinaday.com.au/</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2023)</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Hi Lifetime in a Day Films team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Desiren Photography &amp; Video</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>wedding photo or video</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Cairns</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/desiren_photography_video</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/melbourne.wedding.photography.and.video</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>https://desiren.com.au/</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>missing meta description</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Hi Desiren Photography &amp; Video team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Luminosity Film Studios</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>wedding photo or video</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Cairns</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/luminosity.studios</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/luminosityfilmstudios</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>https://luminosityfilmstudios.com/</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2015)</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Hi Luminosity Film Studios team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Style Productions</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>wedding photo or video</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Cairns</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/styleproductionscairns</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/styleproductionscairns</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.styleproductions.com.au/</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>missing meta description; slow to load (5.1s)</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Hi Style Productions team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Emma G Photos</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Cairns</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/emmagphotographycairns</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/egphotoscairns</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>https://emmagphotos.com/</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>slow to load (5.7s)</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Hi Emma G Photos team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Matthew Evans Photography</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Cairns</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/matthew_evans_photography</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cairnsphotography</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.matthewevansphotography.com.au/</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2015)</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Hi Matthew Evans Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Zen Photography</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Cairns</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/zenphotography_au</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>https://facebook.com/zen.theartofseeing</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.zenphotography.com.au/</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>missing meta description</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Hi Zen Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Clover Studios</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Gold Coast</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/clover__studios</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cloverstudiosphotography</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.clover-studios.com/</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>missing meta description; slow to load (8.7s)</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Hi Clover Studios team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Jennifer McCue Photography</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Hervey Bay</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/jennifermccuephotography</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Jennifer-McCue-Photography-141676235860814</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>https://jennifermccuephotography.com.au/</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>missing meta description</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Hi Jennifer McCue Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Jennifer Treloar Photography</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Mackay</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>https://facebook.com/jennifertreloarphotography</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jennifertreloar.com.au/</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>slow to load (3.3s)</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Hi Jennifer Treloar Photography team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Brisbane Wedding and Lifestyle Photography</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Moreton Bay</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/brisbaneweddingphotography_</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/BrisbaneWeddingPhotographyVideography</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>https://brisbane-photography.com.au/</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>slow to load (5.9s)</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Hi Brisbane Wedding and Lifestyle Photography team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Romana Saeheng Photography</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Redlands</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/RomanaSaeheng</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/RomanaSaeheng</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>https://romana.com.au/</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2018)</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Hi Romana Saeheng Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>All the Love in the World</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Sunshine Coast</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alltheloveintheworld_photos</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/alltheloveintheworldphotography</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>http://www.alltheloveintheworld.com.au/</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>no HTTPS (browser shows 'Not secure')</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Hi All the Love in the World team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Lisa Pearl Photography</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Sunshine Coast</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lisapearlphotography</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/lisapearlphotography</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>https://lisapearl.com.au/</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>missing meta description</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Hi Lisa Pearl Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Neil Hole Wedding Photography</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Sunshine Coast</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/neilholephotography</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/neilholephotography</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>https://neilhole.com.au/</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>slow to load (3.5s)</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Hi Neil Hole Wedding Photography team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Matt Edwards Photography</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Toowoomba</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/matt_edwards_photography_</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/mattedwardsphotography</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>https://mattedwardsphotography.com.au/</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>slow to load (5.5s)</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Hi Matt Edwards Photography team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>The Finches</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Toowoomba</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>http://instagram.com/thefinches</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>http://facebook.com/thefinchesphotography</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>http://www.thefinches.com.au/</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2022)</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Hi The Finches team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Sapphire Soul Photography</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>wedding photo or video</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/sapphiresoulcreative</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sapphiresoul.com.au/</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2023)</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Hi Sapphire Soul Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Beyond the Spectrum Photography</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>wedding photographer</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/beyondthespectrumphotography</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/beyondthespectrumphotography</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>https://beyondthespectrumphotography.com.au/</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2020)</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Hi Beyond the Spectrum Photography team! [one real detail from their page]. We're AceAds, a web design studio. We think your website could be doing more to bring in customers. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Weak website</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>JC Filmz</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>wedding videographer</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/jcfilmz.townsville</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/JCFilmz</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>https://jcfilmz.com/</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>looks outdated (copyright 2019); slow to load (3.9s)</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Hi JC Filmz team! [one real detail from their page]. We're AceAds, a web design studio. We noticed your site loads slowly on a phone, and that's often where couples and clients first see your galleries. We'd be happy to make you a free preview of what a website could look like. Want one? No cost, no obligation.</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S6"/>
-  <conditionalFormatting sqref="A2:S6">
+  <autoFilter ref="A1:S28"/>
+  <conditionalFormatting sqref="A2:S28">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$O2="Won"</formula>
     </cfRule>
@@ -1025,29 +2643,116 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="O2:O6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O2:O28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not contacted,DM sent,Replied,Preview sent,Meeting booked,Won,Not interested,Business closed"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:R6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date"/>
+    <dataValidation sqref="Q2:R28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date"/>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId104"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1059,7 +2764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1067,12 +2772,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
@@ -1172,13 +2877,13 @@
           <t>Reply rate (Replied or later / DMs sent)</t>
         </is>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="6">
         <f>IFERROR((B4+B5+B6+B7+B8)/(B3+B4+B5+B6+B7+B8),0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Leads per priority</t>
         </is>
@@ -1219,7 +2924,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Leads per region</t>
         </is>
@@ -1240,22 +2945,110 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Bundaberg</t>
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF(Leads!F:F,"Ipswich")</f>
+        <f>COUNTIF(Leads!F:F,"Bundaberg")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Cairns</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>COUNTIF(Leads!F:F,"Cairns")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Gold Coast</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>COUNTIF(Leads!F:F,"Gold Coast")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hervey Bay</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>COUNTIF(Leads!F:F,"Hervey Bay")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mackay</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>COUNTIF(Leads!F:F,"Mackay")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Moreton Bay</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>COUNTIF(Leads!F:F,"Moreton Bay")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Redlands</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>COUNTIF(Leads!F:F,"Redlands")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Sunshine Coast</t>
         </is>
       </c>
-      <c r="B20">
+      <c r="B26">
         <f>COUNTIF(Leads!F:F,"Sunshine Coast")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Toowoomba</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>COUNTIF(Leads!F:F,"Toowoomba")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>COUNTIF(Leads!F:F,"Townsville")</f>
         <v/>
       </c>
     </row>
@@ -1277,9 +3070,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>AceAds: Instagram / Facebook outreach, Brisbane, Ipswich, Sunshine Coast</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>AceAds: Instagram / Facebook outreach, Queensland</t>
         </is>
       </c>
     </row>
@@ -1287,7 +3080,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Before each DM</t>
         </is>
@@ -1325,7 +3118,7 @@
       <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Sending</t>
         </is>
@@ -1377,7 +3170,7 @@
       <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Do not</t>
         </is>

</xml_diff>

<commit_message>
Wedding photo/video DM workbook: 27 QLD leads; warn that load times are measured from overseas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xNR6qHipSou6potzqm3UQ
</commit_message>
<xml_diff>
--- a/results/AceAds-DM-outreach-Wedding-Photo-Video-QLD.xlsx
+++ b/results/AceAds-DM-outreach-Wedding-Photo-Video-QLD.xlsx
@@ -3063,7 +3063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -3115,100 +3115,107 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4. 'Slow to load' was timed from an overseas server. Open the site on your own phone first; if it loads fine, skip that point.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Sending</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>4. Send from the AceAds business account, by hand. Max 20 new DMs per account per day.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5. Never paste the identical message twice in a row. Personalise every one; Meta limits accounts that send copy-paste DMs.</t>
+          <t>5. Send from the AceAds business account, by hand. Max 20 new DMs per account per day.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6. If they reply yes, ask AceAds for their preview (mockups/ in the repo), then send the screenshot and link.</t>
+          <t>6. Never paste the identical message twice in a row. Personalise every one; Meta limits accounts that send copy-paste DMs.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Set Status to 'Preview sent'.</t>
+          <t>7. If they reply yes, ask AceAds for their preview (mockups/ in the repo), then send the screenshot and link.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7. One polite follow-up after 4-5 days, only if there was no reply. Then stop.</t>
+          <t xml:space="preserve">   Set Status to 'Preview sent'.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8. If anyone says no or asks us to stop, set 'Not interested' and never contact them again.</t>
+          <t>8. One polite follow-up after 4-5 days, only if there was no reply. Then stop.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9. If anyone says no or asks us to stop, set 'Not interested' and never contact them again.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Do not</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>- Do not add these businesses to bulk email or automated DM tools.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>- Email only to an address the business publishes on its own website, copied by hand. Say who we are, keep it</t>
+          <t>- Do not add these businesses to bulk email or automated DM tools.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  about their website, and end with: 'Not interested? Reply STOP and we won't contact you again.'</t>
+          <t>- Email only to an address the business publishes on its own website, copied by hand. Say who we are, keep it</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t xml:space="preserve">  about their website, and end with: 'Not interested? Reply STOP and we won't contact you again.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>- Do not claim anything about their business you have not checked.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Source: OpenStreetMap (c) OpenStreetMap contributors, plus links found on the businesses' own websites.</t>
         </is>

</xml_diff>